<commit_message>
Bugs corrigidos e pronto para teste em uma base real antes de liberar para produção
</commit_message>
<xml_diff>
--- a/foton_system/foton_make/testes/baseDados.xlsx
+++ b/foton_system/foton_make/testes/baseDados.xlsx
@@ -590,7 +590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -678,36 +678,18 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>LAMP</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>202401001</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Projeto Padrão</t>
-        </is>
-      </c>
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>PROJ-1</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>1042024</v>
-      </c>
-      <c r="F3" t="n">
-        <v>2500</v>
-      </c>
-      <c r="G3" t="n">
-        <v>5000</v>
-      </c>
-      <c r="H3" t="n">
-        <v>1</v>
-      </c>
+          <t>PROJ-2</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
           <t>LUCAS LAMP</t>
@@ -720,14 +702,18 @@
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>CLIENTE-TESTE-1</t>
+          <t>SERVICO-TEST-1</t>
         </is>
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>CLIENTE-TESTE-1</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr"/>
@@ -735,14 +721,18 @@
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>CLIENTE-TESTE-2</t>
+          <t>SERVICO-CL2-TESTE</t>
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>CLIENTE-TESTE-2</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr"/>
@@ -750,69 +740,16 @@
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>LUCAS LAMP</t>
+          <t>PROJ-01-CLIENTE-TESTE-3</t>
         </is>
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>SERVICO-TEST-1</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>CLIENTE-TESTE-1</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr"/>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>SERVICO-CL2-TESTE</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>CLIENTE-TESTE-2</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>PROJ-2</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>LUCAS LAMP</t>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>CLIENTE-TESTE-3</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Aplicação para ler os emails recebidos do cadastro do site e exportar para csv
</commit_message>
<xml_diff>
--- a/foton_system/foton_make/testes/baseDados.xlsx
+++ b/foton_system/foton_make/testes/baseDados.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="1"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="baseClientes"/>
@@ -306,7 +306,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd hh:mm:ss"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -316,19 +316,13 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -341,7 +335,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -371,26 +365,11 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="13">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -401,11 +380,11 @@
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -413,22 +392,13 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -742,27 +712,27 @@
   <dimension ref="A1:E38"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="6" width="14.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="6" width="30.576428571428572" customWidth="1" bestFit="1"/>
     <col min="3" max="3" style="6" width="20.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="14" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="15" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="11" width="17.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="12" width="20.433571428571426" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="20.25">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="8" t="s">
         <v>77</v>
       </c>
     </row>
@@ -776,11 +746,11 @@
       <c r="C2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="11">
+      <c r="D2" s="4">
         <v>3999354100</v>
       </c>
-      <c r="E2" s="12">
-        <v>25568.875295925925</v>
+      <c r="E2" s="9">
+        <v>25568.875300925927</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
@@ -789,8 +759,8 @@
       <c r="C3" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="D3" s="11"/>
-      <c r="E3" s="13"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="3"/>
@@ -798,8 +768,8 @@
       <c r="C4" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="D4" s="11"/>
-      <c r="E4" s="13"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="3"/>
@@ -807,8 +777,8 @@
       <c r="C5" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D5" s="11"/>
-      <c r="E5" s="13"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="3"/>
@@ -816,8 +786,8 @@
       <c r="C6" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="11"/>
-      <c r="E6" s="13"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="3"/>
@@ -825,8 +795,8 @@
       <c r="C7" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="D7" s="11"/>
-      <c r="E7" s="13"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="3"/>
@@ -834,8 +804,8 @@
       <c r="C8" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D8" s="11"/>
-      <c r="E8" s="13"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="3"/>
@@ -843,8 +813,8 @@
       <c r="C9" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="D9" s="11"/>
-      <c r="E9" s="13"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
       <c r="A10" s="3"/>
@@ -852,8 +822,8 @@
       <c r="C10" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="D10" s="11"/>
-      <c r="E10" s="13"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
       <c r="A11" s="3"/>
@@ -861,8 +831,8 @@
       <c r="C11" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="D11" s="11"/>
-      <c r="E11" s="13"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
       <c r="A12" s="3"/>
@@ -870,8 +840,8 @@
       <c r="C12" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="D12" s="11"/>
-      <c r="E12" s="13"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
       <c r="A13" s="3"/>
@@ -879,8 +849,8 @@
       <c r="C13" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="D13" s="11"/>
-      <c r="E13" s="13"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
       <c r="A14" s="3"/>
@@ -888,8 +858,8 @@
       <c r="C14" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="D14" s="11"/>
-      <c r="E14" s="13"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
       <c r="A15" s="3"/>
@@ -897,8 +867,8 @@
       <c r="C15" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D15" s="11"/>
-      <c r="E15" s="13"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
       <c r="A16" s="3"/>
@@ -906,8 +876,8 @@
       <c r="C16" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="D16" s="11"/>
-      <c r="E16" s="13"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
       <c r="A17" s="3"/>
@@ -915,8 +885,8 @@
       <c r="C17" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="D17" s="11"/>
-      <c r="E17" s="13"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
       <c r="A18" s="3"/>
@@ -924,8 +894,8 @@
       <c r="C18" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="D18" s="11"/>
-      <c r="E18" s="13"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
       <c r="A19" s="3"/>
@@ -933,8 +903,8 @@
       <c r="C19" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="D19" s="11"/>
-      <c r="E19" s="13"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
       <c r="A20" s="3"/>
@@ -942,8 +912,8 @@
       <c r="C20" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="D20" s="11"/>
-      <c r="E20" s="13"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
       <c r="A21" s="3"/>
@@ -951,8 +921,8 @@
       <c r="C21" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="D21" s="11"/>
-      <c r="E21" s="13"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
       <c r="A22" s="3"/>
@@ -960,8 +930,8 @@
       <c r="C22" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="D22" s="11"/>
-      <c r="E22" s="13"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
       <c r="A23" s="3"/>
@@ -969,8 +939,8 @@
       <c r="C23" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D23" s="11"/>
-      <c r="E23" s="13"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
       <c r="A24" s="3"/>
@@ -978,8 +948,8 @@
       <c r="C24" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="D24" s="11"/>
-      <c r="E24" s="13"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
       <c r="A25" s="3"/>
@@ -987,8 +957,8 @@
       <c r="C25" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D25" s="11"/>
-      <c r="E25" s="13"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
       <c r="A26" s="3"/>
@@ -996,8 +966,8 @@
       <c r="C26" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="D26" s="11"/>
-      <c r="E26" s="13"/>
+      <c r="D26" s="4"/>
+      <c r="E26" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
       <c r="A27" s="3"/>
@@ -1005,8 +975,8 @@
       <c r="C27" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D27" s="11"/>
-      <c r="E27" s="13"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
       <c r="A28" s="3"/>
@@ -1014,8 +984,8 @@
       <c r="C28" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="D28" s="11"/>
-      <c r="E28" s="13"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
       <c r="A29" s="3"/>
@@ -1023,8 +993,8 @@
       <c r="C29" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="D29" s="11"/>
-      <c r="E29" s="13"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
       <c r="A30" s="3"/>
@@ -1032,8 +1002,8 @@
       <c r="C30" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="D30" s="11"/>
-      <c r="E30" s="13"/>
+      <c r="D30" s="4"/>
+      <c r="E30" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
       <c r="A31" s="3"/>
@@ -1041,8 +1011,8 @@
       <c r="C31" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D31" s="11"/>
-      <c r="E31" s="13"/>
+      <c r="D31" s="4"/>
+      <c r="E31" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
       <c r="A32" s="3"/>
@@ -1050,8 +1020,8 @@
       <c r="C32" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D32" s="11"/>
-      <c r="E32" s="13"/>
+      <c r="D32" s="4"/>
+      <c r="E32" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
       <c r="A33" s="3"/>
@@ -1059,8 +1029,8 @@
       <c r="C33" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="D33" s="11"/>
-      <c r="E33" s="13"/>
+      <c r="D33" s="4"/>
+      <c r="E33" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
       <c r="A34" s="3"/>
@@ -1068,8 +1038,8 @@
       <c r="C34" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="D34" s="11"/>
-      <c r="E34" s="13"/>
+      <c r="D34" s="4"/>
+      <c r="E34" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
       <c r="A35" s="3"/>
@@ -1077,8 +1047,8 @@
       <c r="C35" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D35" s="11"/>
-      <c r="E35" s="13"/>
+      <c r="D35" s="4"/>
+      <c r="E35" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
       <c r="A36" s="3"/>
@@ -1086,8 +1056,8 @@
       <c r="C36" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="D36" s="11"/>
-      <c r="E36" s="13"/>
+      <c r="D36" s="4"/>
+      <c r="E36" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75">
       <c r="A37" s="3"/>
@@ -1095,8 +1065,8 @@
       <c r="C37" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D37" s="11"/>
-      <c r="E37" s="13"/>
+      <c r="D37" s="4"/>
+      <c r="E37" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75">
       <c r="A38" s="3"/>
@@ -1104,8 +1074,8 @@
       <c r="C38" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="D38" s="11"/>
-      <c r="E38" s="13"/>
+      <c r="D38" s="4"/>
+      <c r="E38" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1131,7 +1101,7 @@
     <col min="9" max="9" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="21">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="20.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1160,7 +1130,7 @@
         <v>8</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="3" t="s">
         <v>9</v>
       </c>

</xml_diff>

<commit_message>
Correção da ferramenta de sincronização do cadastro no email
</commit_message>
<xml_diff>
--- a/foton_system/foton_make/testes/baseDados.xlsx
+++ b/foton_system/foton_make/testes/baseDados.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="96">
   <si>
     <t>CodCliente</t>
   </si>
@@ -245,10 +245,16 @@
     <t>NomeCliente</t>
   </si>
   <si>
-    <t>CpfCliente</t>
-  </si>
-  <si>
     <t>NasCliente</t>
+  </si>
+  <si>
+    <t>CpfCnpjCliente</t>
+  </si>
+  <si>
+    <t>TelefoneCLiente</t>
+  </si>
+  <si>
+    <t>EmailCliente</t>
   </si>
   <si>
     <t>Lucas Antonio Magalhães Pereira</t>
@@ -306,7 +312,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd hh:mm:ss"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -317,12 +323,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -369,7 +369,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -383,14 +383,11 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -398,11 +395,11 @@
     <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
     <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -709,14 +706,16 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="6" width="14.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="6" width="30.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="6" width="20.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="11" width="17.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="12" width="20.433571428571426" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="5" width="14.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="5" width="30.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="5" width="20.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="6" width="17.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="5" width="20.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="11" width="20.433571428571426" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="20.25">
@@ -732,8 +731,14 @@
       <c r="D1" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="2" t="s">
         <v>77</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>79</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
@@ -741,260 +746,320 @@
         <v>9</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="8">
+        <v>25568.375300925927</v>
+      </c>
+      <c r="E2" s="4">
         <v>3999354100</v>
       </c>
-      <c r="E2" s="9">
+      <c r="F2" s="9">
+        <v>5562981613868</v>
+      </c>
+      <c r="G2" s="8">
         <v>25568.875300925927</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3" t="s">
         <v>54</v>
       </c>
       <c r="D3" s="4"/>
-      <c r="E3" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="10"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="3"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D4" s="4"/>
-      <c r="E4" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="10"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3" t="s">
         <v>27</v>
       </c>
       <c r="D5" s="4"/>
-      <c r="E5" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="10"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3" t="s">
         <v>17</v>
       </c>
       <c r="D6" s="4"/>
-      <c r="E6" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="10"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
       <c r="A7" s="3"/>
       <c r="B7" s="3"/>
       <c r="C7" s="3" t="s">
         <v>59</v>
       </c>
       <c r="D7" s="4"/>
-      <c r="E7" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="10"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
       <c r="A8" s="3"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3" t="s">
         <v>45</v>
       </c>
       <c r="D8" s="4"/>
-      <c r="E8" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="10"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
       <c r="A9" s="3"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3" t="s">
         <v>49</v>
       </c>
       <c r="D9" s="4"/>
-      <c r="E9" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="10"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
       <c r="A10" s="3"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D10" s="4"/>
-      <c r="E10" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="10"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3" t="s">
         <v>73</v>
       </c>
       <c r="D11" s="4"/>
-      <c r="E11" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="10"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
       <c r="A12" s="3"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3" t="s">
         <v>29</v>
       </c>
       <c r="D12" s="4"/>
-      <c r="E12" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="10"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3" t="s">
         <v>31</v>
       </c>
       <c r="D13" s="4"/>
-      <c r="E13" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="10"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="C14" s="3" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D14" s="4"/>
-      <c r="E14" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="10"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3" t="s">
         <v>24</v>
       </c>
       <c r="D15" s="4"/>
-      <c r="E15" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="10"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D16" s="4"/>
-      <c r="E16" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="10"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5">
       <c r="A17" s="3"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D17" s="4"/>
-      <c r="E17" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="10"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
       <c r="A18" s="3"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D18" s="4"/>
-      <c r="E18" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="10"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5">
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D19" s="4"/>
-      <c r="E19" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="10"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="19.5">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
       <c r="C20" s="3" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D20" s="4"/>
-      <c r="E20" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="10"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="19.5">
       <c r="A21" s="3"/>
       <c r="B21" s="3"/>
       <c r="C21" s="3" t="s">
         <v>40</v>
       </c>
       <c r="D21" s="4"/>
-      <c r="E21" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="10"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="19.5">
       <c r="A22" s="3"/>
       <c r="B22" s="3"/>
       <c r="C22" s="3" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D22" s="4"/>
-      <c r="E22" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="10"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="19.5">
       <c r="A23" s="3"/>
       <c r="B23" s="3"/>
       <c r="C23" s="3" t="s">
         <v>43</v>
       </c>
       <c r="D23" s="4"/>
-      <c r="E23" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="10"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="19.5">
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
       <c r="C24" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D24" s="4"/>
-      <c r="E24" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="10"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="19.5">
       <c r="A25" s="3"/>
       <c r="B25" s="3"/>
       <c r="C25" s="3" t="s">
         <v>38</v>
       </c>
       <c r="D25" s="4"/>
-      <c r="E25" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="10"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="19.5">
       <c r="A26" s="3"/>
       <c r="B26" s="3"/>
       <c r="C26" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D26" s="4"/>
-      <c r="E26" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
+      <c r="G26" s="10"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="19.5">
       <c r="A27" s="3"/>
       <c r="B27" s="3"/>
       <c r="C27" s="3" t="s">
         <v>47</v>
       </c>
       <c r="D27" s="4"/>
-      <c r="E27" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
+      <c r="E27" s="3"/>
+      <c r="F27" s="3"/>
+      <c r="G27" s="10"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="19.5">
       <c r="A28" s="3"/>
       <c r="B28" s="3"/>
       <c r="C28" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D28" s="4"/>
-      <c r="E28" s="10"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="10"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="19.5">
       <c r="A29" s="3"/>
       <c r="B29" s="3"/>
       <c r="C29" s="3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D29" s="4"/>
-      <c r="E29" s="10"/>
+      <c r="E29" s="3"/>
+      <c r="F29" s="3"/>
+      <c r="G29" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
       <c r="A30" s="3"/>
@@ -1003,7 +1068,9 @@
         <v>56</v>
       </c>
       <c r="D30" s="4"/>
-      <c r="E30" s="10"/>
+      <c r="E30" s="3"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
       <c r="A31" s="3"/>
@@ -1012,7 +1079,9 @@
         <v>19</v>
       </c>
       <c r="D31" s="4"/>
-      <c r="E31" s="10"/>
+      <c r="E31" s="3"/>
+      <c r="F31" s="3"/>
+      <c r="G31" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
       <c r="A32" s="3"/>
@@ -1021,7 +1090,9 @@
         <v>22</v>
       </c>
       <c r="D32" s="4"/>
-      <c r="E32" s="10"/>
+      <c r="E32" s="3"/>
+      <c r="F32" s="3"/>
+      <c r="G32" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
       <c r="A33" s="3"/>
@@ -1030,16 +1101,20 @@
         <v>71</v>
       </c>
       <c r="D33" s="4"/>
-      <c r="E33" s="10"/>
+      <c r="E33" s="3"/>
+      <c r="F33" s="3"/>
+      <c r="G33" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
       <c r="A34" s="3"/>
       <c r="B34" s="3"/>
       <c r="C34" s="3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D34" s="4"/>
-      <c r="E34" s="10"/>
+      <c r="E34" s="3"/>
+      <c r="F34" s="3"/>
+      <c r="G34" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
       <c r="A35" s="3"/>
@@ -1048,7 +1123,9 @@
         <v>33</v>
       </c>
       <c r="D35" s="4"/>
-      <c r="E35" s="10"/>
+      <c r="E35" s="3"/>
+      <c r="F35" s="3"/>
+      <c r="G35" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
       <c r="A36" s="3"/>
@@ -1057,7 +1134,9 @@
         <v>61</v>
       </c>
       <c r="D36" s="4"/>
-      <c r="E36" s="10"/>
+      <c r="E36" s="3"/>
+      <c r="F36" s="3"/>
+      <c r="G36" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75">
       <c r="A37" s="3"/>
@@ -1066,16 +1145,20 @@
         <v>14</v>
       </c>
       <c r="D37" s="4"/>
-      <c r="E37" s="10"/>
+      <c r="E37" s="3"/>
+      <c r="F37" s="3"/>
+      <c r="G37" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75">
       <c r="A38" s="3"/>
       <c r="B38" s="3"/>
       <c r="C38" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D38" s="4"/>
-      <c r="E38" s="10"/>
+      <c r="E38" s="3"/>
+      <c r="F38" s="3"/>
+      <c r="G38" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1090,15 +1173,15 @@
   <dimension ref="A1:I42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="6" width="19.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="5" width="19.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="20.25">
@@ -1161,600 +1244,600 @@
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="3"/>
-      <c r="B3" s="5"/>
+      <c r="B3" s="4"/>
       <c r="C3" s="3"/>
       <c r="D3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
       <c r="I3" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="3"/>
-      <c r="B4" s="5"/>
+      <c r="B4" s="4"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
       <c r="I4" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="3"/>
-      <c r="B5" s="5"/>
+      <c r="B5" s="4"/>
       <c r="C5" s="3"/>
       <c r="D5" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
+      <c r="H5" s="4"/>
       <c r="I5" s="3" t="s">
         <v>17</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="3"/>
-      <c r="B6" s="5"/>
+      <c r="B6" s="4"/>
       <c r="C6" s="3"/>
       <c r="D6" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="4"/>
+      <c r="H6" s="4"/>
       <c r="I6" s="3" t="s">
         <v>19</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="3"/>
-      <c r="B7" s="5"/>
+      <c r="B7" s="4"/>
       <c r="C7" s="3"/>
       <c r="D7" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="4"/>
+      <c r="H7" s="4"/>
       <c r="I7" s="3" t="s">
         <v>19</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="3"/>
-      <c r="B8" s="5"/>
+      <c r="B8" s="4"/>
       <c r="C8" s="3"/>
       <c r="D8" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
+      <c r="G8" s="4"/>
+      <c r="H8" s="4"/>
       <c r="I8" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="3"/>
-      <c r="B9" s="5"/>
+      <c r="B9" s="4"/>
       <c r="C9" s="3"/>
       <c r="D9" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="4"/>
+      <c r="H9" s="4"/>
       <c r="I9" s="3" t="s">
         <v>24</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
       <c r="A10" s="3"/>
-      <c r="B10" s="5"/>
+      <c r="B10" s="4"/>
       <c r="C10" s="3"/>
       <c r="D10" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="4"/>
+      <c r="H10" s="4"/>
       <c r="I10" s="3" t="s">
         <v>24</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
       <c r="A11" s="3"/>
-      <c r="B11" s="5"/>
+      <c r="B11" s="4"/>
       <c r="C11" s="3"/>
       <c r="D11" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="4"/>
+      <c r="H11" s="4"/>
       <c r="I11" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
       <c r="A12" s="3"/>
-      <c r="B12" s="5"/>
+      <c r="B12" s="4"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="5"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="4"/>
+      <c r="H12" s="4"/>
       <c r="I12" s="3" t="s">
         <v>29</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
       <c r="A13" s="3"/>
-      <c r="B13" s="5"/>
+      <c r="B13" s="4"/>
       <c r="C13" s="3"/>
       <c r="D13" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
       <c r="I13" s="3" t="s">
         <v>31</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
       <c r="A14" s="3"/>
-      <c r="B14" s="5"/>
+      <c r="B14" s="4"/>
       <c r="C14" s="3"/>
       <c r="D14" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="4"/>
+      <c r="H14" s="4"/>
       <c r="I14" s="3" t="s">
         <v>33</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
       <c r="A15" s="3"/>
-      <c r="B15" s="5"/>
+      <c r="B15" s="4"/>
       <c r="C15" s="3"/>
       <c r="D15" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="5"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="4"/>
+      <c r="G15" s="4"/>
+      <c r="H15" s="4"/>
       <c r="I15" s="3" t="s">
         <v>33</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
       <c r="A16" s="3"/>
-      <c r="B16" s="5"/>
+      <c r="B16" s="4"/>
       <c r="C16" s="3"/>
       <c r="D16" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
-      <c r="H16" s="5"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="4"/>
+      <c r="G16" s="4"/>
+      <c r="H16" s="4"/>
       <c r="I16" s="3" t="s">
         <v>33</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
       <c r="A17" s="3"/>
-      <c r="B17" s="5"/>
+      <c r="B17" s="4"/>
       <c r="C17" s="3"/>
       <c r="D17" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="E17" s="5"/>
-      <c r="F17" s="5"/>
-      <c r="G17" s="5"/>
-      <c r="H17" s="5"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="4"/>
+      <c r="G17" s="4"/>
+      <c r="H17" s="4"/>
       <c r="I17" s="3" t="s">
         <v>33</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
       <c r="A18" s="3"/>
-      <c r="B18" s="5"/>
+      <c r="B18" s="4"/>
       <c r="C18" s="3"/>
       <c r="D18" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
-      <c r="G18" s="5"/>
-      <c r="H18" s="5"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="4"/>
+      <c r="H18" s="4"/>
       <c r="I18" s="3" t="s">
         <v>38</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
       <c r="A19" s="3"/>
-      <c r="B19" s="5"/>
+      <c r="B19" s="4"/>
       <c r="C19" s="3"/>
       <c r="D19" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4"/>
+      <c r="G19" s="4"/>
+      <c r="H19" s="4"/>
       <c r="I19" s="3" t="s">
         <v>40</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
       <c r="A20" s="3"/>
-      <c r="B20" s="5"/>
+      <c r="B20" s="4"/>
       <c r="C20" s="3"/>
       <c r="D20" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4"/>
+      <c r="G20" s="4"/>
+      <c r="H20" s="4"/>
       <c r="I20" s="3" t="s">
         <v>40</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
       <c r="A21" s="3"/>
-      <c r="B21" s="5"/>
+      <c r="B21" s="4"/>
       <c r="C21" s="3"/>
       <c r="D21" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
-      <c r="H21" s="5"/>
+      <c r="E21" s="4"/>
+      <c r="F21" s="4"/>
+      <c r="G21" s="4"/>
+      <c r="H21" s="4"/>
       <c r="I21" s="3" t="s">
         <v>43</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
       <c r="A22" s="3"/>
-      <c r="B22" s="5"/>
+      <c r="B22" s="4"/>
       <c r="C22" s="3"/>
       <c r="D22" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
-      <c r="G22" s="5"/>
-      <c r="H22" s="5"/>
+      <c r="E22" s="4"/>
+      <c r="F22" s="4"/>
+      <c r="G22" s="4"/>
+      <c r="H22" s="4"/>
       <c r="I22" s="3" t="s">
         <v>45</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
       <c r="A23" s="3"/>
-      <c r="B23" s="5"/>
+      <c r="B23" s="4"/>
       <c r="C23" s="3"/>
       <c r="D23" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="E23" s="5"/>
-      <c r="F23" s="5"/>
-      <c r="G23" s="5"/>
-      <c r="H23" s="5"/>
+      <c r="E23" s="4"/>
+      <c r="F23" s="4"/>
+      <c r="G23" s="4"/>
+      <c r="H23" s="4"/>
       <c r="I23" s="3" t="s">
         <v>47</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
       <c r="A24" s="3"/>
-      <c r="B24" s="5"/>
+      <c r="B24" s="4"/>
       <c r="C24" s="3"/>
       <c r="D24" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="E24" s="5"/>
-      <c r="F24" s="5"/>
-      <c r="G24" s="5"/>
-      <c r="H24" s="5"/>
+      <c r="E24" s="4"/>
+      <c r="F24" s="4"/>
+      <c r="G24" s="4"/>
+      <c r="H24" s="4"/>
       <c r="I24" s="3" t="s">
         <v>49</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
       <c r="A25" s="3"/>
-      <c r="B25" s="5"/>
+      <c r="B25" s="4"/>
       <c r="C25" s="3"/>
       <c r="D25" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="E25" s="5"/>
-      <c r="F25" s="5"/>
-      <c r="G25" s="5"/>
-      <c r="H25" s="5"/>
+      <c r="E25" s="4"/>
+      <c r="F25" s="4"/>
+      <c r="G25" s="4"/>
+      <c r="H25" s="4"/>
       <c r="I25" s="3" t="s">
         <v>49</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
       <c r="A26" s="3"/>
-      <c r="B26" s="5"/>
+      <c r="B26" s="4"/>
       <c r="C26" s="3"/>
       <c r="D26" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="E26" s="5"/>
-      <c r="F26" s="5"/>
-      <c r="G26" s="5"/>
-      <c r="H26" s="5"/>
+      <c r="E26" s="4"/>
+      <c r="F26" s="4"/>
+      <c r="G26" s="4"/>
+      <c r="H26" s="4"/>
       <c r="I26" s="3" t="s">
         <v>49</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
       <c r="A27" s="3"/>
-      <c r="B27" s="5"/>
+      <c r="B27" s="4"/>
       <c r="C27" s="3"/>
       <c r="D27" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="E27" s="5"/>
-      <c r="F27" s="5"/>
-      <c r="G27" s="5"/>
-      <c r="H27" s="5"/>
+      <c r="E27" s="4"/>
+      <c r="F27" s="4"/>
+      <c r="G27" s="4"/>
+      <c r="H27" s="4"/>
       <c r="I27" s="3" t="s">
         <v>49</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
       <c r="A28" s="3"/>
-      <c r="B28" s="5"/>
+      <c r="B28" s="4"/>
       <c r="C28" s="3"/>
       <c r="D28" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="E28" s="5"/>
-      <c r="F28" s="5"/>
-      <c r="G28" s="5"/>
-      <c r="H28" s="5"/>
+      <c r="E28" s="4"/>
+      <c r="F28" s="4"/>
+      <c r="G28" s="4"/>
+      <c r="H28" s="4"/>
       <c r="I28" s="3" t="s">
         <v>54</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
       <c r="A29" s="3"/>
-      <c r="B29" s="5"/>
+      <c r="B29" s="4"/>
       <c r="C29" s="3"/>
       <c r="D29" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="E29" s="5"/>
-      <c r="F29" s="5"/>
-      <c r="G29" s="5"/>
-      <c r="H29" s="5"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+      <c r="G29" s="4"/>
+      <c r="H29" s="4"/>
       <c r="I29" s="3" t="s">
         <v>56</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
       <c r="A30" s="3"/>
-      <c r="B30" s="5"/>
+      <c r="B30" s="4"/>
       <c r="C30" s="3"/>
       <c r="D30" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="E30" s="5"/>
-      <c r="F30" s="5"/>
-      <c r="G30" s="5"/>
-      <c r="H30" s="5"/>
+      <c r="E30" s="4"/>
+      <c r="F30" s="4"/>
+      <c r="G30" s="4"/>
+      <c r="H30" s="4"/>
       <c r="I30" s="3" t="s">
         <v>56</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
       <c r="A31" s="3"/>
-      <c r="B31" s="5"/>
+      <c r="B31" s="4"/>
       <c r="C31" s="3"/>
       <c r="D31" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="E31" s="5"/>
-      <c r="F31" s="5"/>
-      <c r="G31" s="5"/>
-      <c r="H31" s="5"/>
+      <c r="E31" s="4"/>
+      <c r="F31" s="4"/>
+      <c r="G31" s="4"/>
+      <c r="H31" s="4"/>
       <c r="I31" s="3" t="s">
         <v>59</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
       <c r="A32" s="3"/>
-      <c r="B32" s="5"/>
+      <c r="B32" s="4"/>
       <c r="C32" s="3"/>
       <c r="D32" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="E32" s="5"/>
-      <c r="F32" s="5"/>
-      <c r="G32" s="5"/>
-      <c r="H32" s="5"/>
+      <c r="E32" s="4"/>
+      <c r="F32" s="4"/>
+      <c r="G32" s="4"/>
+      <c r="H32" s="4"/>
       <c r="I32" s="3" t="s">
         <v>61</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
       <c r="A33" s="3"/>
-      <c r="B33" s="5"/>
+      <c r="B33" s="4"/>
       <c r="C33" s="3"/>
       <c r="D33" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="E33" s="5"/>
-      <c r="F33" s="5"/>
-      <c r="G33" s="5"/>
-      <c r="H33" s="5"/>
+      <c r="E33" s="4"/>
+      <c r="F33" s="4"/>
+      <c r="G33" s="4"/>
+      <c r="H33" s="4"/>
       <c r="I33" s="3" t="s">
         <v>61</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
       <c r="A34" s="3"/>
-      <c r="B34" s="5"/>
+      <c r="B34" s="4"/>
       <c r="C34" s="3"/>
       <c r="D34" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="E34" s="5"/>
-      <c r="F34" s="5"/>
-      <c r="G34" s="5"/>
-      <c r="H34" s="5"/>
+      <c r="E34" s="4"/>
+      <c r="F34" s="4"/>
+      <c r="G34" s="4"/>
+      <c r="H34" s="4"/>
       <c r="I34" s="3" t="s">
         <v>61</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
       <c r="A35" s="3"/>
-      <c r="B35" s="5"/>
+      <c r="B35" s="4"/>
       <c r="C35" s="3"/>
       <c r="D35" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="E35" s="5"/>
-      <c r="F35" s="5"/>
-      <c r="G35" s="5"/>
-      <c r="H35" s="5"/>
+      <c r="E35" s="4"/>
+      <c r="F35" s="4"/>
+      <c r="G35" s="4"/>
+      <c r="H35" s="4"/>
       <c r="I35" s="3" t="s">
         <v>61</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
       <c r="A36" s="3"/>
-      <c r="B36" s="5"/>
+      <c r="B36" s="4"/>
       <c r="C36" s="3"/>
       <c r="D36" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="E36" s="5"/>
-      <c r="F36" s="5"/>
-      <c r="G36" s="5"/>
-      <c r="H36" s="5"/>
+      <c r="E36" s="4"/>
+      <c r="F36" s="4"/>
+      <c r="G36" s="4"/>
+      <c r="H36" s="4"/>
       <c r="I36" s="3" t="s">
         <v>61</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75">
       <c r="A37" s="3"/>
-      <c r="B37" s="5"/>
+      <c r="B37" s="4"/>
       <c r="C37" s="3"/>
       <c r="D37" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="E37" s="5"/>
-      <c r="F37" s="5"/>
-      <c r="G37" s="5"/>
-      <c r="H37" s="5"/>
+      <c r="E37" s="4"/>
+      <c r="F37" s="4"/>
+      <c r="G37" s="4"/>
+      <c r="H37" s="4"/>
       <c r="I37" s="3" t="s">
         <v>61</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75">
       <c r="A38" s="3"/>
-      <c r="B38" s="5"/>
+      <c r="B38" s="4"/>
       <c r="C38" s="3"/>
       <c r="D38" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="E38" s="5"/>
-      <c r="F38" s="5"/>
-      <c r="G38" s="5"/>
-      <c r="H38" s="5"/>
+      <c r="E38" s="4"/>
+      <c r="F38" s="4"/>
+      <c r="G38" s="4"/>
+      <c r="H38" s="4"/>
       <c r="I38" s="3" t="s">
         <v>61</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75">
       <c r="A39" s="3"/>
-      <c r="B39" s="5"/>
+      <c r="B39" s="4"/>
       <c r="C39" s="3"/>
       <c r="D39" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="E39" s="5"/>
-      <c r="F39" s="5"/>
-      <c r="G39" s="5"/>
-      <c r="H39" s="5"/>
+      <c r="E39" s="4"/>
+      <c r="F39" s="4"/>
+      <c r="G39" s="4"/>
+      <c r="H39" s="4"/>
       <c r="I39" s="3" t="s">
         <v>61</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18.75">
       <c r="A40" s="3"/>
-      <c r="B40" s="5"/>
+      <c r="B40" s="4"/>
       <c r="C40" s="3"/>
       <c r="D40" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="E40" s="5"/>
-      <c r="F40" s="5"/>
-      <c r="G40" s="5"/>
-      <c r="H40" s="5"/>
+      <c r="E40" s="4"/>
+      <c r="F40" s="4"/>
+      <c r="G40" s="4"/>
+      <c r="H40" s="4"/>
       <c r="I40" s="3" t="s">
         <v>61</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75">
       <c r="A41" s="3"/>
-      <c r="B41" s="5"/>
+      <c r="B41" s="4"/>
       <c r="C41" s="3"/>
       <c r="D41" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="E41" s="5"/>
-      <c r="F41" s="5"/>
-      <c r="G41" s="5"/>
-      <c r="H41" s="5"/>
+      <c r="E41" s="4"/>
+      <c r="F41" s="4"/>
+      <c r="G41" s="4"/>
+      <c r="H41" s="4"/>
       <c r="I41" s="3" t="s">
         <v>71</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18.75">
       <c r="A42" s="3"/>
-      <c r="B42" s="5"/>
+      <c r="B42" s="4"/>
       <c r="C42" s="3"/>
       <c r="D42" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="E42" s="5"/>
-      <c r="F42" s="5"/>
-      <c r="G42" s="5"/>
-      <c r="H42" s="5"/>
+      <c r="E42" s="4"/>
+      <c r="F42" s="4"/>
+      <c r="G42" s="4"/>
+      <c r="H42" s="4"/>
       <c r="I42" s="3" t="s">
         <v>73</v>
       </c>

</xml_diff>